<commit_message>
data(characters): G01-P7-C04 import character partition 04
</commit_message>
<xml_diff>
--- a/config/data/AbilityHitPlanBinding.xlsx
+++ b/config/data/AbilityHitPlanBinding.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J169"/>
+  <dimension ref="A1:J199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12.7109375" customWidth="1" min="1" max="1"/>
@@ -5055,6 +5055,936 @@
       <c r="H169" t="inlineStr">
         <is>
           <t>Quantum</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="B170" t="n">
+        <v>60002</v>
+      </c>
+      <c r="C170" t="n">
+        <v>1</v>
+      </c>
+      <c r="D170" t="n">
+        <v>61001</v>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>parameter.01</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>Atk</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>Ordinary</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>Fire</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="B171" t="n">
+        <v>60005</v>
+      </c>
+      <c r="C171" t="n">
+        <v>1</v>
+      </c>
+      <c r="D171" t="n">
+        <v>61002</v>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>parameter.01</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>Atk</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>Ordinary</t>
+        </is>
+      </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>Fire</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="B172" t="n">
+        <v>60006</v>
+      </c>
+      <c r="C172" t="n">
+        <v>1</v>
+      </c>
+      <c r="D172" t="n">
+        <v>61003</v>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>parameter.01</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>Atk</t>
+        </is>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>Ordinary</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>Fire</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="B173" t="n">
+        <v>60008</v>
+      </c>
+      <c r="C173" t="n">
+        <v>1</v>
+      </c>
+      <c r="D173" t="n">
+        <v>61004</v>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>parameter.02</t>
+        </is>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>Atk</t>
+        </is>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>Ordinary</t>
+        </is>
+      </c>
+      <c r="H173" t="inlineStr">
+        <is>
+          <t>Fire</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="B174" t="n">
+        <v>60010</v>
+      </c>
+      <c r="C174" t="n">
+        <v>1</v>
+      </c>
+      <c r="D174" t="n">
+        <v>61005</v>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>parameter.01</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>Atk</t>
+        </is>
+      </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>Ordinary</t>
+        </is>
+      </c>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>Fire</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="B175" t="n">
+        <v>60011</v>
+      </c>
+      <c r="C175" t="n">
+        <v>1</v>
+      </c>
+      <c r="D175" t="n">
+        <v>61006</v>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>parameter.01</t>
+        </is>
+      </c>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>Atk</t>
+        </is>
+      </c>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>Ordinary</t>
+        </is>
+      </c>
+      <c r="H175" t="inlineStr">
+        <is>
+          <t>Fire</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="B176" t="n">
+        <v>60012</v>
+      </c>
+      <c r="C176" t="n">
+        <v>1</v>
+      </c>
+      <c r="D176" t="n">
+        <v>61007</v>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>parameter.01</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>Atk</t>
+        </is>
+      </c>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>Ordinary</t>
+        </is>
+      </c>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>Fire</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="B177" t="n">
+        <v>60017</v>
+      </c>
+      <c r="C177" t="n">
+        <v>1</v>
+      </c>
+      <c r="D177" t="n">
+        <v>61008</v>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>parameter.01</t>
+        </is>
+      </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>Atk</t>
+        </is>
+      </c>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>Ordinary</t>
+        </is>
+      </c>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>Ice</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="B178" t="n">
+        <v>60019</v>
+      </c>
+      <c r="C178" t="n">
+        <v>1</v>
+      </c>
+      <c r="D178" t="n">
+        <v>61009</v>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>parameter.01</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>Atk</t>
+        </is>
+      </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>Ordinary</t>
+        </is>
+      </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>Ice</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="B179" t="n">
+        <v>60022</v>
+      </c>
+      <c r="C179" t="n">
+        <v>1</v>
+      </c>
+      <c r="D179" t="n">
+        <v>61010</v>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>parameter.01</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>Atk</t>
+        </is>
+      </c>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>Ordinary</t>
+        </is>
+      </c>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>Fire</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="B180" t="n">
+        <v>60024</v>
+      </c>
+      <c r="C180" t="n">
+        <v>1</v>
+      </c>
+      <c r="D180" t="n">
+        <v>61011</v>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>parameter.01</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>Atk</t>
+        </is>
+      </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>Ordinary</t>
+        </is>
+      </c>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>Fire</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="B181" t="n">
+        <v>60025</v>
+      </c>
+      <c r="C181" t="n">
+        <v>1</v>
+      </c>
+      <c r="D181" t="n">
+        <v>61012</v>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>parameter.01</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>Atk</t>
+        </is>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>Ordinary</t>
+        </is>
+      </c>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>Fire</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="B182" t="n">
+        <v>60026</v>
+      </c>
+      <c r="C182" t="n">
+        <v>1</v>
+      </c>
+      <c r="D182" t="n">
+        <v>61013</v>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>parameter.01</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>Atk</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>Ordinary</t>
+        </is>
+      </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>Fire</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="B183" t="n">
+        <v>60029</v>
+      </c>
+      <c r="C183" t="n">
+        <v>1</v>
+      </c>
+      <c r="D183" t="n">
+        <v>61014</v>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>parameter.01</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr">
+        <is>
+          <t>Atk</t>
+        </is>
+      </c>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>Ordinary</t>
+        </is>
+      </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>Physical</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="B184" t="n">
+        <v>60030</v>
+      </c>
+      <c r="C184" t="n">
+        <v>1</v>
+      </c>
+      <c r="D184" t="n">
+        <v>61015</v>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>parameter.01</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr">
+        <is>
+          <t>Atk</t>
+        </is>
+      </c>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>Ordinary</t>
+        </is>
+      </c>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>Physical</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="B185" t="n">
+        <v>60034</v>
+      </c>
+      <c r="C185" t="n">
+        <v>1</v>
+      </c>
+      <c r="D185" t="n">
+        <v>61016</v>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>parameter.01</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>Atk</t>
+        </is>
+      </c>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>Ordinary</t>
+        </is>
+      </c>
+      <c r="H185" t="inlineStr">
+        <is>
+          <t>Ice</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="B186" t="n">
+        <v>60036</v>
+      </c>
+      <c r="C186" t="n">
+        <v>1</v>
+      </c>
+      <c r="D186" t="n">
+        <v>61017</v>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>parameter.01</t>
+        </is>
+      </c>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>Atk</t>
+        </is>
+      </c>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>Ordinary</t>
+        </is>
+      </c>
+      <c r="H186" t="inlineStr">
+        <is>
+          <t>Ice</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="B187" t="n">
+        <v>60037</v>
+      </c>
+      <c r="C187" t="n">
+        <v>1</v>
+      </c>
+      <c r="D187" t="n">
+        <v>61018</v>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>parameter.01</t>
+        </is>
+      </c>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>Atk</t>
+        </is>
+      </c>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>Ordinary</t>
+        </is>
+      </c>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>Ice</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="B188" t="n">
+        <v>60038</v>
+      </c>
+      <c r="C188" t="n">
+        <v>1</v>
+      </c>
+      <c r="D188" t="n">
+        <v>61019</v>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>parameter.01</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>Atk</t>
+        </is>
+      </c>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t>Ordinary</t>
+        </is>
+      </c>
+      <c r="H188" t="inlineStr">
+        <is>
+          <t>Ice</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="B189" t="n">
+        <v>60040</v>
+      </c>
+      <c r="C189" t="n">
+        <v>1</v>
+      </c>
+      <c r="D189" t="n">
+        <v>61020</v>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>parameter.01</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>Atk</t>
+        </is>
+      </c>
+      <c r="G189" t="inlineStr">
+        <is>
+          <t>Ordinary</t>
+        </is>
+      </c>
+      <c r="H189" t="inlineStr">
+        <is>
+          <t>Fire</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="B190" t="n">
+        <v>60041</v>
+      </c>
+      <c r="C190" t="n">
+        <v>1</v>
+      </c>
+      <c r="D190" t="n">
+        <v>61021</v>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>parameter.01</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>Atk</t>
+        </is>
+      </c>
+      <c r="G190" t="inlineStr">
+        <is>
+          <t>Ordinary</t>
+        </is>
+      </c>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>Fire</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="B191" t="n">
+        <v>60042</v>
+      </c>
+      <c r="C191" t="n">
+        <v>1</v>
+      </c>
+      <c r="D191" t="n">
+        <v>61022</v>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>parameter.01</t>
+        </is>
+      </c>
+      <c r="F191" t="inlineStr">
+        <is>
+          <t>Atk</t>
+        </is>
+      </c>
+      <c r="G191" t="inlineStr">
+        <is>
+          <t>Ordinary</t>
+        </is>
+      </c>
+      <c r="H191" t="inlineStr">
+        <is>
+          <t>Fire</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="B192" t="n">
+        <v>60043</v>
+      </c>
+      <c r="C192" t="n">
+        <v>1</v>
+      </c>
+      <c r="D192" t="n">
+        <v>61023</v>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>parameter.01</t>
+        </is>
+      </c>
+      <c r="F192" t="inlineStr">
+        <is>
+          <t>Atk</t>
+        </is>
+      </c>
+      <c r="G192" t="inlineStr">
+        <is>
+          <t>Ordinary</t>
+        </is>
+      </c>
+      <c r="H192" t="inlineStr">
+        <is>
+          <t>Fire</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="B193" t="n">
+        <v>60045</v>
+      </c>
+      <c r="C193" t="n">
+        <v>1</v>
+      </c>
+      <c r="D193" t="n">
+        <v>61024</v>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>parameter.01</t>
+        </is>
+      </c>
+      <c r="F193" t="inlineStr">
+        <is>
+          <t>Atk</t>
+        </is>
+      </c>
+      <c r="G193" t="inlineStr">
+        <is>
+          <t>Ordinary</t>
+        </is>
+      </c>
+      <c r="H193" t="inlineStr">
+        <is>
+          <t>Fire</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="B194" t="n">
+        <v>60047</v>
+      </c>
+      <c r="C194" t="n">
+        <v>1</v>
+      </c>
+      <c r="D194" t="n">
+        <v>61025</v>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>parameter.01</t>
+        </is>
+      </c>
+      <c r="F194" t="inlineStr">
+        <is>
+          <t>Atk</t>
+        </is>
+      </c>
+      <c r="G194" t="inlineStr">
+        <is>
+          <t>Ordinary</t>
+        </is>
+      </c>
+      <c r="H194" t="inlineStr">
+        <is>
+          <t>Fire</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="B195" t="n">
+        <v>60049</v>
+      </c>
+      <c r="C195" t="n">
+        <v>1</v>
+      </c>
+      <c r="D195" t="n">
+        <v>61026</v>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>parameter.01</t>
+        </is>
+      </c>
+      <c r="F195" t="inlineStr">
+        <is>
+          <t>Atk</t>
+        </is>
+      </c>
+      <c r="G195" t="inlineStr">
+        <is>
+          <t>Ordinary</t>
+        </is>
+      </c>
+      <c r="H195" t="inlineStr">
+        <is>
+          <t>Fire</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="B196" t="n">
+        <v>60051</v>
+      </c>
+      <c r="C196" t="n">
+        <v>1</v>
+      </c>
+      <c r="D196" t="n">
+        <v>61027</v>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>parameter.01</t>
+        </is>
+      </c>
+      <c r="F196" t="inlineStr">
+        <is>
+          <t>Atk</t>
+        </is>
+      </c>
+      <c r="G196" t="inlineStr">
+        <is>
+          <t>Ordinary</t>
+        </is>
+      </c>
+      <c r="H196" t="inlineStr">
+        <is>
+          <t>Fire</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="B197" t="n">
+        <v>60053</v>
+      </c>
+      <c r="C197" t="n">
+        <v>1</v>
+      </c>
+      <c r="D197" t="n">
+        <v>61028</v>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>parameter.01</t>
+        </is>
+      </c>
+      <c r="F197" t="inlineStr">
+        <is>
+          <t>Atk</t>
+        </is>
+      </c>
+      <c r="G197" t="inlineStr">
+        <is>
+          <t>Ordinary</t>
+        </is>
+      </c>
+      <c r="H197" t="inlineStr">
+        <is>
+          <t>Fire</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="B198" t="n">
+        <v>60054</v>
+      </c>
+      <c r="C198" t="n">
+        <v>1</v>
+      </c>
+      <c r="D198" t="n">
+        <v>61029</v>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>parameter.01</t>
+        </is>
+      </c>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>Atk</t>
+        </is>
+      </c>
+      <c r="G198" t="inlineStr">
+        <is>
+          <t>Ordinary</t>
+        </is>
+      </c>
+      <c r="H198" t="inlineStr">
+        <is>
+          <t>Fire</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="B199" t="n">
+        <v>60055</v>
+      </c>
+      <c r="C199" t="n">
+        <v>1</v>
+      </c>
+      <c r="D199" t="n">
+        <v>61030</v>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>parameter.01</t>
+        </is>
+      </c>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>Atk</t>
+        </is>
+      </c>
+      <c r="G199" t="inlineStr">
+        <is>
+          <t>Ordinary</t>
+        </is>
+      </c>
+      <c r="H199" t="inlineStr">
+        <is>
+          <t>Fire</t>
         </is>
       </c>
     </row>

</xml_diff>